<commit_message>
Fill HSK1_parts_of_speech_3(101-150).xlsx with parts of speech
</commit_message>
<xml_diff>
--- a/HSK1_parts_of_speech_3(101-150).xlsx
+++ b/HSK1_parts_of_speech_3(101-150).xlsx
@@ -601,6 +601,11 @@
           <t>комната</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>комната</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -632,6 +637,11 @@
           <t>да</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>дом, здание</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -658,6 +668,11 @@
           <t>отпускать</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>класть, ставить; отпускать; выпускать (журнал)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -684,6 +699,16 @@
           <t>отпускать на каникулы</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>уходить на каникулы/выходные</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>словосочетание (离合词: 放…假)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -710,6 +735,16 @@
           <t>закончить занятия</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>заканчивать занятия (в школе)</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>словосочетание (离合词: 放…学)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -736,6 +771,16 @@
           <t>летать</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>летать</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>быстрый (разг. 飞块)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -762,6 +807,11 @@
           <t>самолёт</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>самолёт</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -788,6 +838,11 @@
           <t>очень</t>
         </is>
       </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>очень, чрезвычайно</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -814,6 +869,21 @@
           <t>минута (счётное слово)</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>минута</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>делить, раздваивать (分开)</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>для деления, частей; для оценок (三分)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -840,6 +910,11 @@
           <t>ветер</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ветер</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -866,6 +941,16 @@
           <t>сухой</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>тофу (豆腐干)</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>сухой</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -892,6 +977,11 @@
           <t>чистый</t>
         </is>
       </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>чистый, опрятный</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -918,6 +1008,16 @@
           <t>делать, заниматься</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>делать, заниматься</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>сильный, крепкий (手脚干); сухое (вино)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -944,6 +1044,11 @@
           <t>Что делать?</t>
         </is>
       </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>вопросительная конструкция «что делаешь? / зачем?»</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -970,6 +1075,11 @@
           <t>высокий</t>
         </is>
       </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>высокий (рост, здания, температура)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -996,6 +1106,11 @@
           <t>радостный</t>
         </is>
       </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>радостный, довольный</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1022,6 +1137,11 @@
           <t>сказать</t>
         </is>
       </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>сообщать, рассказывать (кому-л.)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1053,6 +1173,11 @@
           <t>старший брат</t>
         </is>
       </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>старший брат</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1079,6 +1204,11 @@
           <t>песня</t>
         </is>
       </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>песня, песенная часть opera</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1105,6 +1235,11 @@
           <t>штука (универсальное счётное слово)</t>
         </is>
       </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>универсальное счётное слово (для большинства предметов, людей, событий)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1131,6 +1266,16 @@
           <t>давать</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>давать, передавать</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>для (кого-л.), кому (给他买)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1157,6 +1302,21 @@
           <t>с, вместе с</t>
         </is>
       </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>следовать, идти за</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>с, вместе с (跟朋友去)</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>и, а также (跟…一样)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1183,6 +1343,11 @@
           <t>рабочий</t>
         </is>
       </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>рабочий, рабочий класс</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1209,6 +1374,16 @@
           <t>работа</t>
         </is>
       </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>работа</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>работать</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1235,6 +1410,11 @@
           <t>закрывать, выключать</t>
         </is>
       </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>закрывать, выключать; иметь отношение (有关)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1261,6 +1441,16 @@
           <t>закрыть, выключить</t>
         </is>
       </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>закрыть, выключить (результат)</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>глагол + результативное дополнение (关上)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1287,6 +1477,11 @@
           <t>дорогой; уважаемый</t>
         </is>
       </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>дорогой (по цене); почтенный, уважаемый (贵姓)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1313,6 +1508,16 @@
           <t>страна, государство; национальный</t>
         </is>
       </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>страна, государство</t>
+        </is>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>национальный (国货, 中文)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1339,6 +1544,11 @@
           <t>страна</t>
         </is>
       </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>страна, государство</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1365,6 +1575,16 @@
           <t>иностранный, зарубежный; вне страны</t>
         </is>
       </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>за границей, за рубежом</t>
+        </is>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>иностранный, зарубежный (国外新闻)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1391,6 +1611,16 @@
           <t>проходить (мимо)</t>
         </is>
       </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>проходить (мимо); пересекать; проходить (о времени)</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>частица опыта (去过, 吃过)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1417,6 +1647,11 @@
           <t>ещё</t>
         </is>
       </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>ещё, всё ещё; всё-таки (还是)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1443,6 +1678,16 @@
           <t>всё-таки, всё еще; или</t>
         </is>
       </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>всё-таки, всё ещё</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>или (в вопросах с выбором)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1469,6 +1714,16 @@
           <t>ещё есть, в дополнение</t>
         </is>
       </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>и ещё, в добавление</t>
+        </is>
+      </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>устойчивое выражение (还有+дополнение)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1500,6 +1755,11 @@
           <t>да</t>
         </is>
       </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>ребёнок, дети</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1526,6 +1786,11 @@
           <t>китайский язык</t>
         </is>
       </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>китайский язык</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1552,6 +1817,11 @@
           <t>китайский иероглиф</t>
         </is>
       </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>китайский иероглиф</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1578,6 +1848,16 @@
           <t>хороший</t>
         </is>
       </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>хороший, добрый</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>почти (好几年), едва не (差点儿没…)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1604,6 +1884,11 @@
           <t>вкусный</t>
         </is>
       </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>вкусный</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1630,6 +1915,11 @@
           <t>красивый</t>
         </is>
       </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>красивый,好看的 (на вид)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1656,6 +1946,11 @@
           <t>приятный для слуха</t>
         </is>
       </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>приятный на слух, благозвучный</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1682,6 +1977,11 @@
           <t>весёлый, интересный</t>
         </is>
       </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>весёлый, интересный, забавный</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1708,6 +2008,16 @@
           <t>номер, дата</t>
         </is>
       </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>номер; число (дата) 十号</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>для дат и номеров</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1734,6 +2044,11 @@
           <t>пить</t>
         </is>
       </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>пить</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1760,6 +2075,21 @@
           <t>и</t>
         </is>
       </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>гармония, мир (和平)</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>с, вместе с (他和我说)</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>и, с (连接 однородные члены)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1786,6 +2116,11 @@
           <t>очень</t>
         </is>
       </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>очень</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1812,6 +2147,21 @@
           <t>позади; после</t>
         </is>
       </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>зад, тыл;后面</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>после (放学后)</t>
+        </is>
+      </c>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>последующий, задний (后年, 后天)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1838,6 +2188,11 @@
           <t>сзади, позади</t>
         </is>
       </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>зад, тыл (方位词)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1864,6 +2219,11 @@
           <t>послезавтра</t>
         </is>
       </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>послезавтра</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1888,6 +2248,16 @@
       <c r="I51" t="inlineStr">
         <is>
           <t>цветок</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>цветок</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>тратить, расходовать (花钱)</t>
         </is>
       </c>
     </row>

</xml_diff>